<commit_message>
fix: range stamp duty algorithm update and rebuild
</commit_message>
<xml_diff>
--- a/files/九龙-启德-The Henley II.xlsx
+++ b/files/九龙-启德-The Henley II.xlsx
@@ -16253,7 +16253,7 @@
         </is>
       </c>
       <c r="E250" s="4" t="n">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F250" s="3" t="inlineStr">
         <is>
@@ -16262,14 +16262,14 @@
       </c>
       <c r="G250" s="3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H250" s="5" t="n">
         <v>17560800</v>
       </c>
       <c r="I250" s="5" t="n">
-        <v>32400</v>
+        <v>32340</v>
       </c>
       <c r="J250" s="3" t="inlineStr">
         <is>
@@ -16280,7 +16280,7 @@
         <v>17560800</v>
       </c>
       <c r="L250" s="5" t="n">
-        <v>32400</v>
+        <v>32340</v>
       </c>
       <c r="M250" s="3" t="inlineStr">
         <is>
@@ -16324,7 +16324,7 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H251" s="5" t="n">
@@ -16819,7 +16819,7 @@
         </is>
       </c>
       <c r="E259" s="4" t="n">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F259" s="3" t="inlineStr">
         <is>
@@ -16828,14 +16828,14 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="H259" s="5" t="n">
         <v>17040000</v>
       </c>
       <c r="I259" s="5" t="n">
-        <v>31439</v>
+        <v>31381</v>
       </c>
       <c r="J259" s="3" t="inlineStr">
         <is>
@@ -16846,7 +16846,7 @@
         <v>17040000</v>
       </c>
       <c r="L259" s="5" t="n">
-        <v>31439</v>
+        <v>31381</v>
       </c>
       <c r="M259" s="3" t="inlineStr">
         <is>
@@ -22014,15 +22014,15 @@
           <t>B | 550呎 (2房)
 $1754万
 $31,900/呎
-(26年-06月-09日)</t>
+(26年-07月-13日)</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>C | 542呎 (2房)
+          <t>C | 543呎 (2房)
 $1756万
-$32,400/呎
-(26年-06月-09日)</t>
+$32,340/呎
+(26年-07月-13日)</t>
         </is>
       </c>
       <c r="E32" s="22" t="inlineStr">
@@ -22098,10 +22098,10 @@
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>C | 542呎 (2房)
+          <t>C | 543呎 (2房)
 $1704万
-$31,439/呎
-(26年-06月-10日)</t>
+$31,381/呎
+(26年-07月-13日)</t>
         </is>
       </c>
       <c r="E33" s="22" t="inlineStr">

</xml_diff>